<commit_message>
update TC Wave 6 + update skill
</commit_message>
<xml_diff>
--- a/practices/testcases/gara-wave06/ui/TC_PRC.xlsx
+++ b/practices/testcases/gara-wave06/ui/TC_PRC.xlsx
@@ -482,7 +482,7 @@
         <v>High</v>
       </c>
       <c r="D3" t="str">
-        <v>Mở màn khi đã có log tính giá</v>
+        <v>Kiểm tra hiển thị màn PRC-LIST thành công với dữ liệu đã có log tính giá</v>
       </c>
       <c r="E3" t="str">
         <v>Tenant có ≥1 log PRC đã chạy</v>
@@ -514,7 +514,7 @@
         <v>High</v>
       </c>
       <c r="D4" t="str">
-        <v>Mở màn khi chưa có log nào (empty state)</v>
+        <v>Kiểm tra hiển thị empty state thành công tại PRC-LIST khi chưa có log nào</v>
       </c>
       <c r="E4" t="str">
         <v>Tenant mới, chưa từng chạy PRC</v>
@@ -544,7 +544,7 @@
         <v>High</v>
       </c>
       <c r="D5" t="str">
-        <v>Nhiều log cùng (kỳ+kho) hiển thị riêng biệt</v>
+        <v>Kiểm tra hiển thị 2 dòng riêng biệt thành công với dữ liệu 2 log cùng (kỳ+kho)</v>
       </c>
       <c r="E5" t="str">
         <v>Đã chạy Tính giá 2 lần cho cùng Kỳ+Kho</v>
@@ -573,7 +573,7 @@
         <v>High</v>
       </c>
       <c r="D6" t="str">
-        <v>Bấm "Xem" điều hướng đúng Detail</v>
+        <v>Kiểm tra điều hướng sang màn Detail thành công khi bấm icon "Xem"</v>
       </c>
       <c r="E6" t="str">
         <v>Bảng có dòng id=4521</v>
@@ -603,7 +603,7 @@
         <v>High</v>
       </c>
       <c r="D7" t="str">
-        <v>Bấm CTA "Tính giá" điều hướng sang Create</v>
+        <v>Kiểm tra điều hướng sang màn Create thành công khi bấm CTA "Tính giá"</v>
       </c>
       <c r="E7" t="str">
         <v>—</v>
@@ -632,7 +632,7 @@
         <v>High</v>
       </c>
       <c r="D8" t="str">
-        <v>Bấm icon "Xóa" mở đúng dialog xác nhận</v>
+        <v>Kiểm tra mở dialog xác nhận xóa thành công khi bấm icon "Xóa"</v>
       </c>
       <c r="E8" t="str">
         <v>Bảng có ≥1 dòng</v>
@@ -661,7 +661,7 @@
         <v>High</v>
       </c>
       <c r="D9" t="str">
-        <v>Lỗi tải danh sách (network/500)</v>
+        <v>Kiểm tra hiển thị lỗi tải danh sách thất bại với dữ liệu BE trả network/500</v>
       </c>
       <c r="E9" t="str">
         <v>Giả lập BE trả lỗi 500</v>
@@ -691,7 +691,7 @@
         <v>High</v>
       </c>
       <c r="D10" t="str">
-        <v>Xóa log đã bị user khác xóa trước (ERR-CMN-not-found)</v>
+        <v>Kiểm tra xóa log thất bại với dữ liệu log đã bị user khác xóa trước (ERR-CMN-not-found)</v>
       </c>
       <c r="E10" t="str">
         <v>2 user cùng mở LIST, user B xóa trước</v>
@@ -752,7 +752,7 @@
         <v>Medium</v>
       </c>
       <c r="D12" t="str">
-        <v>Filter "Ngày thực hiện" — executedFrom &gt; executedTo</v>
+        <v>Kiểm tra validate filter "Ngày thực hiện" thất bại khi executedFrom &gt; executedTo</v>
       </c>
       <c r="E12" t="str">
         <v>Bảng có data nhiều ngày</v>
@@ -783,7 +783,7 @@
         <v>Medium</v>
       </c>
       <c r="D13" t="str">
-        <v>Filter "Ngày thực hiện" — khoảng hợp lệ</v>
+        <v>Kiểm tra filter "Ngày thực hiện" thành công với khoảng ngày hợp lệ</v>
       </c>
       <c r="E13" t="str">
         <v>Bảng có data trong khoảng</v>
@@ -814,7 +814,7 @@
         <v>Medium</v>
       </c>
       <c r="D14" t="str">
-        <v>Filter "Phương pháp" — chỉ có 1 option</v>
+        <v>Kiểm tra hiển thị dropdown filter "Phương pháp" thành công với dữ liệu chỉ có 1 option</v>
       </c>
       <c r="E14" t="str">
         <v>—</v>
@@ -844,7 +844,7 @@
         <v>Medium</v>
       </c>
       <c r="D15" t="str">
-        <v>Kết hợp cả 2 filter (AND)</v>
+        <v>Kiểm tra kết hợp 2 filter "Phương pháp" + "Ngày thực hiện" thành công theo điều kiện AND</v>
       </c>
       <c r="E15" t="str">
         <v>Data đa dạng</v>
@@ -902,7 +902,7 @@
         <v>Medium</v>
       </c>
       <c r="D17" t="str">
-        <v>Badge trạng thái đúng 3 màu/nhãn</v>
+        <v>Kiểm tra hiển thị đúng badge trạng thái với dữ liệu 3 log ở 3 trạng thái khác nhau</v>
       </c>
       <c r="E17" t="str">
         <v>3 log ở 3 trạng thái khác nhau</v>
@@ -933,7 +933,7 @@
         <v>Low</v>
       </c>
       <c r="D18" t="str">
-        <v>Semantic HTML — heading &amp; table header</v>
+        <v>Kiểm tra semantic HTML đúng chuẩn cho heading và table header tại PRC-LIST</v>
       </c>
       <c r="E18" t="str">
         <v>—</v>
@@ -963,7 +963,7 @@
         <v>Low</v>
       </c>
       <c r="D19" t="str">
-        <v>Icon action có aria-label</v>
+        <v>Kiểm tra icon action Xem/Xóa có đúng thuộc tính aria-label</v>
       </c>
       <c r="E19" t="str">
         <v>Bảng có data</v>
@@ -993,7 +993,7 @@
         <v>Medium</v>
       </c>
       <c r="D20" t="str">
-        <v>Empty state đúng test-id và text verbatim</v>
+        <v>Kiểm tra hiển thị empty state đúng test-id và text verbatim khi chưa có log</v>
       </c>
       <c r="E20" t="str">
         <v>Tenant chưa có log</v>
@@ -1023,7 +1023,7 @@
         <v>Medium</v>
       </c>
       <c r="D21" t="str">
-        <v>Pagination — đổi page-size reset về trang 0</v>
+        <v>Kiểm tra pagination reset về trang 0 thành công khi đổi page-size với dữ liệu ≥25 dòng</v>
       </c>
       <c r="E21" t="str">
         <v>≥25 dòng data</v>
@@ -1054,7 +1054,7 @@
         <v>Low</v>
       </c>
       <c r="D22" t="str">
-        <v>Loading state dùng skeleton bảng</v>
+        <v>Kiểm tra hiển thị loading state dạng skeleton bảng khi PRC-LIST đang tải</v>
       </c>
       <c r="E22" t="str">
         <v>—</v>
@@ -1084,7 +1084,7 @@
         <v>Low</v>
       </c>
       <c r="D23" t="str">
-        <v>Tab order đúng thứ tự DOM</v>
+        <v>Kiểm tra tab order đúng thứ tự DOM tại màn PRC-LIST</v>
       </c>
       <c r="E23" t="str">
         <v>—</v>
@@ -1113,7 +1113,7 @@
         <v>Low</v>
       </c>
       <c r="D24" t="str">
-        <v>Confirm dialog xóa — focus-trap &amp; focus trả về</v>
+        <v>Kiểm tra focus-trap và focus trả về đúng thành công khi thao tác dialog xác nhận xóa</v>
       </c>
       <c r="E24" t="str">
         <v>Bảng có data</v>
@@ -1174,7 +1174,7 @@
         <v>High</v>
       </c>
       <c r="D26" t="str">
-        <v>garage-owner truy cập đầy đủ quyền</v>
+        <v>Kiểm tra phân quyền truy cập đầy đủ thành công cho vai trò garage-owner tại PRC-LIST</v>
       </c>
       <c r="E26" t="str">
         <v>Tài khoản garage-owner</v>
@@ -1204,7 +1204,7 @@
         <v>High</v>
       </c>
       <c r="D27" t="str">
-        <v>accountant truy cập đầy đủ quyền</v>
+        <v>Kiểm tra phân quyền truy cập đầy đủ thành công cho vai trò accountant tại PRC-LIST</v>
       </c>
       <c r="E27" t="str">
         <v>Tài khoản accountant</v>
@@ -1234,7 +1234,7 @@
         <v>High</v>
       </c>
       <c r="D28" t="str">
-        <v>Feature flag OFF</v>
+        <v>Kiểm tra chặn truy cập route PRC-LIST thành công khi feature flag Inventory:InventoryV2 đang OFF</v>
       </c>
       <c r="E28" t="str">
         <v>Tenant chưa bật Inventory:InventoryV2</v>
@@ -1292,7 +1292,7 @@
         <v>High</v>
       </c>
       <c r="D30" t="str">
-        <v>Sau CREATE, LIST hiện dòng mới đầu bảng</v>
+        <v>Kiểm tra LIST cập nhật đúng dòng mới ở đầu bảng thành công sau khi CREATE</v>
       </c>
       <c r="E30" t="str">
         <v>Vừa tạo 1 lần tính mới ở M2</v>
@@ -1321,7 +1321,7 @@
         <v>High</v>
       </c>
       <c r="D31" t="str">
-        <v>Sau DELETE (không phải dòng cuối trang)</v>
+        <v>Kiểm tra LIST cập nhật đúng thành công sau khi xóa 1 dòng không phải dòng cuối trang</v>
       </c>
       <c r="E31" t="str">
         <v>Trang có 20 dòng, xóa 1 dòng giữa</v>
@@ -1350,7 +1350,7 @@
         <v>High</v>
       </c>
       <c r="D32" t="str">
-        <v>Xóa dòng cuối trang → tự lùi trang</v>
+        <v>Kiểm tra LIST tự động lùi trang thành công khi xóa dòng duy nhất của trang cuối</v>
       </c>
       <c r="E32" t="str">
         <v>Trang cuối chỉ còn 1 dòng</v>
@@ -1379,7 +1379,7 @@
         <v>High</v>
       </c>
       <c r="D33" t="str">
-        <v>Sau RECALC, LIST hiện cả log cũ lẫn mới</v>
+        <v>Kiểm tra LIST hiển thị đúng cả log cũ lẫn mới thành công sau khi RECALC</v>
       </c>
       <c r="E33" t="str">
         <v>Đã RECALC 1 log</v>
@@ -1437,7 +1437,7 @@
         <v>High</v>
       </c>
       <c r="D35" t="str">
-        <v>Mở form từ CTA "Tính giá"</v>
+        <v>Kiểm tra mở form CREATE thành công khi bấm CTA "Tính giá"</v>
       </c>
       <c r="E35" t="str">
         <v>—</v>
@@ -1467,7 +1467,7 @@
         <v>High</v>
       </c>
       <c r="D36" t="str">
-        <v>Chọn Kỳ kế toán → tự khóa Từ/Đến ngày</v>
+        <v>Kiểm tra tự động khóa Từ ngày/Đến ngày thành công khi chọn Kỳ kế toán "Tháng 07/2026"</v>
       </c>
       <c r="E36" t="str">
         <v>Kỳ "Tháng 07/2026" tồn tại</v>
@@ -1497,7 +1497,7 @@
         <v>High</v>
       </c>
       <c r="D37" t="str">
-        <v>Chọn Kho + Phương pháp mặc định</v>
+        <v>Kiểm tra tự động chọn Phương pháp mặc định thành công khi chọn Kho</v>
       </c>
       <c r="E37" t="str">
         <v>—</v>
@@ -1526,7 +1526,7 @@
         <v>High</v>
       </c>
       <c r="D38" t="str">
-        <v>Chọn "Tất cả mã" → ẩn bảng vật tư</v>
+        <v>Kiểm tra ẩn bảng vật tư thành công khi chọn Phạm vi vật tư = "Tất cả mã"</v>
       </c>
       <c r="E38" t="str">
         <v>—</v>
@@ -1556,7 +1556,7 @@
         <v>High</v>
       </c>
       <c r="D39" t="str">
-        <v>Chọn "Chọn mã cụ thể" → hiện bảng vật tư</v>
+        <v>Kiểm tra hiển thị bảng vật tư thành công khi chọn Phạm vi vật tư = "Chọn mã cụ thể"</v>
       </c>
       <c r="E39" t="str">
         <v>—</v>
@@ -1585,7 +1585,7 @@
         <v>High</v>
       </c>
       <c r="D40" t="str">
-        <v>Thêm 1 dòng, chọn mã hợp lệ</v>
+        <v>Kiểm tra thêm dòng vật tư thành công với mã nội bộ hợp lệ PN-18901</v>
       </c>
       <c r="E40" t="str">
         <v>Scope = Chọn mã cụ thể</v>
@@ -1616,7 +1616,7 @@
         <v>High</v>
       </c>
       <c r="D41" t="str">
-        <v>Xóa 1 dòng đã thêm (chưa submit)</v>
+        <v>Kiểm tra xóa dòng vật tư thành công với dữ liệu dòng vừa thêm chưa submit</v>
       </c>
       <c r="E41" t="str">
         <v>Đã thêm ≥1 dòng</v>
@@ -1645,7 +1645,7 @@
         <v>High</v>
       </c>
       <c r="D42" t="str">
-        <v>Submit "Tất cả mã" thành công</v>
+        <v>Kiểm tra submit CREATE thành công với Phạm vi vật tư = "Tất cả mã"</v>
       </c>
       <c r="E42" t="str">
         <v>Kỳ mở, Kho hợp lệ</v>
@@ -1676,7 +1676,7 @@
         <v>High</v>
       </c>
       <c r="D43" t="str">
-        <v>Submit "Chọn mã cụ thể" với 3 mã</v>
+        <v>Kiểm tra submit CREATE thành công với Phạm vi vật tư = "Chọn mã cụ thể" và dữ liệu 3 mã</v>
       </c>
       <c r="E43" t="str">
         <v>Kỳ mở, đã thêm 3 mã hợp lệ</v>
@@ -1705,7 +1705,7 @@
         <v>High</v>
       </c>
       <c r="D44" t="str">
-        <v>CREATE cho kỳ N dù kỳ N-1 chưa từng tính giá</v>
+        <v>Kiểm tra submit CREATE thành công cho kỳ N với dữ liệu kỳ N-1 chưa từng tính giá</v>
       </c>
       <c r="E44" t="str">
         <v>Kỳ N-1 "Tháng 06/2026" chưa có log PRC nào; Kỳ N "Tháng 07/2026" mở</v>
@@ -1736,7 +1736,7 @@
         <v>High</v>
       </c>
       <c r="D45" t="str">
-        <v>Double-click Submit liên tiếp</v>
+        <v>Kiểm tra chặn tạo trùng job thành công khi double-click nút Submit liên tiếp</v>
       </c>
       <c r="E45" t="str">
         <v>Form hợp lệ</v>
@@ -1766,7 +1766,7 @@
         <v>High</v>
       </c>
       <c r="D46" t="str">
-        <v>Submit "Chọn mã cụ thể" nhưng bảng rỗng</v>
+        <v>Kiểm tra chặn submit CREATE thất bại khi Phạm vi = "Chọn mã cụ thể" nhưng bảng vật tư rỗng</v>
       </c>
       <c r="E46" t="str">
         <v>Scope=SPECIFIC, chưa thêm dòng nào</v>
@@ -1795,7 +1795,7 @@
         <v>High</v>
       </c>
       <c r="D47" t="str">
-        <v>Submit khi kỳ đã đóng</v>
+        <v>Kiểm tra submit CREATE thất bại với dữ liệu Kỳ kế toán đã đóng</v>
       </c>
       <c r="E47" t="str">
         <v>Kỳ "Tháng 06/2026" đã đóng</v>
@@ -1826,7 +1826,7 @@
         <v>High</v>
       </c>
       <c r="D48" t="str">
-        <v>Submit khi đã có job chạy cùng kỳ+kho</v>
+        <v>Kiểm tra submit CREATE thất bại khi đã có job PENDING chạy cùng kỳ+kho</v>
       </c>
       <c r="E48" t="str">
         <v>Đang có 1 job PENDING cùng (kỳ, kho)</v>
@@ -1856,7 +1856,7 @@
         <v>High</v>
       </c>
       <c r="D49" t="str">
-        <v>Response có affectedSubsequentPeriods</v>
+        <v>Kiểm tra hiển thị toast cảnh báo thành công với dữ liệu response có affectedSubsequentPeriods</v>
       </c>
       <c r="E49" t="str">
         <v>Kỳ sau đã có log tính trước</v>
@@ -1886,7 +1886,7 @@
         <v>High</v>
       </c>
       <c r="D50" t="str">
-        <v>Bấm "Hủy bỏ"</v>
+        <v>Kiểm tra hủy form CREATE thành công khi bấm nút "Huỷ bỏ"</v>
       </c>
       <c r="E50" t="str">
         <v>—</v>
@@ -1945,7 +1945,7 @@
         <v>Medium</v>
       </c>
       <c r="D52" t="str">
-        <v>Field "Kỳ kế toán" — để trống</v>
+        <v>Kiểm tra validate field "Kỳ kế toán" thất bại khi để trống</v>
       </c>
       <c r="E52" t="str">
         <v>—</v>
@@ -1975,7 +1975,7 @@
         <v>Medium</v>
       </c>
       <c r="D53" t="str">
-        <v>Field "Kho" — để trống</v>
+        <v>Kiểm tra validate field "Kho" thất bại khi để trống</v>
       </c>
       <c r="E53" t="str">
         <v>Đã chọn Kỳ</v>
@@ -2005,7 +2005,7 @@
         <v>Medium</v>
       </c>
       <c r="D54" t="str">
-        <v>Field "Phạm vi vật tư" — chưa chọn</v>
+        <v>Kiểm tra validate field "Phạm vi vật tư" thất bại khi chưa chọn</v>
       </c>
       <c r="E54" t="str">
         <v>—</v>
@@ -2035,7 +2035,7 @@
         <v>Medium</v>
       </c>
       <c r="D55" t="str">
-        <v>Dropdown "Mã nội bộ" — search đúng, chỉ hiện mã BQGQ "Đang hoạt động"</v>
+        <v>Kiểm tra dropdown "Mã nội bộ" search thành công chỉ trả về mã BQGQ "Đang hoạt động" với từ khóa "PN-189"</v>
       </c>
       <c r="E55" t="str">
         <v>Có mã PN-18901(Đang HĐ, BQGQ) và PN-18902(Ngừng HĐ)</v>
@@ -2065,7 +2065,7 @@
         <v>Medium</v>
       </c>
       <c r="D56" t="str">
-        <v>Dropdown "Mã nội bộ" — search không khớp</v>
+        <v>Kiểm tra dropdown "Mã nội bộ" search rỗng thành công với từ khóa không khớp "XYZ-99999"</v>
       </c>
       <c r="E56" t="str">
         <v>—</v>
@@ -2094,7 +2094,7 @@
         <v>Medium</v>
       </c>
       <c r="D57" t="str">
-        <v>Thêm 2 dòng cùng chọn 1 mã trùng nhau</v>
+        <v>Kiểm tra validate chặn trùng mã thành công khi thêm 2 dòng cùng chọn mã PN-18901</v>
       </c>
       <c r="E57" t="str">
         <v>Scope=SPECIFIC</v>
@@ -2104,7 +2104,7 @@
 2. Thêm dòng 2, chọn lại PN-18901</v>
       </c>
       <c r="G57" t="str">
-        <v>1. Ghi nhận hành vi thực tế (spec chưa quy định rõ có chặn trùng hay không) — NEED CONFIRMATION nếu BE không tự loại trùng</v>
+        <v>1. Dòng 2 báo lỗi inline "Mã đã được chọn" ngay khi chọn, KHÔNG cho thêm trùng vào bảng [ASSUMPTION: PTTK không quy định rõ hành vi — chọn chặn trùng phía client vì bảng vật tư là state cục bộ trước khi submit; xác nhận lại với BA/dev nếu BE cũng cần validate trùng khi submit]</v>
       </c>
       <c r="H57" t="str">
         <v>Low</v>
@@ -2153,7 +2153,7 @@
         <v>Medium</v>
       </c>
       <c r="D59" t="str">
-        <v>Input ngày disabled vẫn có label liên kết</v>
+        <v>Kiểm tra input ngày disabled vẫn giữ đúng label liên kết</v>
       </c>
       <c r="E59" t="str">
         <v>Đã chọn Kỳ</v>
@@ -2183,7 +2183,7 @@
         <v>Medium</v>
       </c>
       <c r="D60" t="str">
-        <v>Label "Huỷ bỏ" đúng verbatim Figma</v>
+        <v>Kiểm tra hiển thị đúng label "Huỷ bỏ" verbatim theo Figma</v>
       </c>
       <c r="E60" t="str">
         <v>—</v>
@@ -2212,7 +2212,7 @@
         <v>Medium</v>
       </c>
       <c r="D61" t="str">
-        <v>Bảng vật tư đúng 7 cột</v>
+        <v>Kiểm tra hiển thị đúng 7 cột bảng vật tư với dữ liệu Phạm vi = "Chọn mã cụ thể"</v>
       </c>
       <c r="E61" t="str">
         <v>Scope=SPECIFIC</v>
@@ -2241,7 +2241,7 @@
         <v>Medium</v>
       </c>
       <c r="D62" t="str">
-        <v>Nút Submit loading state</v>
+        <v>Kiểm tra hiển thị loading state thành công cho nút Submit với dữ liệu form hợp lệ</v>
       </c>
       <c r="E62" t="str">
         <v>Form hợp lệ</v>
@@ -2270,7 +2270,7 @@
         <v>Medium</v>
       </c>
       <c r="D63" t="str">
-        <v>Dòng mới thêm — icon xóa ẩn cho tới khi có mã hợp lệ</v>
+        <v>Kiểm tra ẩn icon xóa thành công cho dòng vật tư mới thêm chưa chọn mã</v>
       </c>
       <c r="E63" t="str">
         <v>Scope=SPECIFIC</v>
@@ -2299,7 +2299,7 @@
         <v>Medium</v>
       </c>
       <c r="D64" t="str">
-        <v>Tab order đúng</v>
+        <v>Kiểm tra tab order đúng thứ tự DOM tại form CREATE</v>
       </c>
       <c r="E64" t="str">
         <v>—</v>
@@ -2357,7 +2357,7 @@
         <v>High</v>
       </c>
       <c r="D66" t="str">
-        <v>garage-owner thấy đầy đủ trường + nút</v>
+        <v>Kiểm tra phân quyền hiển thị đầy đủ trường và nút thành công cho vai trò garage-owner tại form CREATE</v>
       </c>
       <c r="E66" t="str">
         <v>Tài khoản garage-owner</v>
@@ -2387,7 +2387,7 @@
         <v>High</v>
       </c>
       <c r="D67" t="str">
-        <v>accountant thấy đầy đủ trường + nút</v>
+        <v>Kiểm tra phân quyền hiển thị đầy đủ trường và nút thành công cho vai trò accountant tại form CREATE</v>
       </c>
       <c r="E67" t="str">
         <v>Tài khoản accountant</v>
@@ -2446,7 +2446,7 @@
         <v>High</v>
       </c>
       <c r="D69" t="str">
-        <v>Sau Submit, LIST hiện log mới đầu bảng đúng trạng thái "Đang tính"</v>
+        <v>Kiểm tra LIST cập nhật đúng log mới với trạng thái "Đang tính" thành công sau khi Submit CREATE</v>
       </c>
       <c r="E69" t="str">
         <v>Vừa Submit thành công</v>
@@ -2475,7 +2475,7 @@
         <v>High</v>
       </c>
       <c r="D70" t="str">
-        <v>Sau khi job hoàn tất, báo cáo Stock V2 cùng mã/kho/kỳ phản ánh đúng</v>
+        <v>Kiểm tra báo cáo Stock V2 cập nhật đúng GT tồn/GT xuất thành công sau khi job PRC hoàn tất</v>
       </c>
       <c r="E70" t="str">
         <v>Job SUCCEEDED</v>
@@ -2533,7 +2533,7 @@
         <v>High</v>
       </c>
       <c r="D72" t="str">
-        <v>Mở từ LIST (click 1 dòng)</v>
+        <v>Kiểm tra mở màn Detail thành công khi click 1 dòng tại LIST</v>
       </c>
       <c r="E72" t="str">
         <v>Bảng LIST có data</v>
@@ -2562,7 +2562,7 @@
         <v>High</v>
       </c>
       <c r="D73" t="str">
-        <v>Mở qua deep-link</v>
+        <v>Kiểm tra mở màn Detail thành công qua deep-link từ toast cảnh báo RECALC</v>
       </c>
       <c r="E73" t="str">
         <v>Có toast cảnh báo từ RECALC chứa link</v>
@@ -2591,7 +2591,7 @@
         <v>High</v>
       </c>
       <c r="D74" t="str">
-        <v>RunInfoGrid hiển thị đúng 8 trường</v>
+        <v>Kiểm tra hiển thị đúng 8 trường tại RunInfoGrid với dữ liệu run đã load</v>
       </c>
       <c r="E74" t="str">
         <v>Run đã load</v>
@@ -2621,7 +2621,7 @@
         <v>High</v>
       </c>
       <c r="D75" t="str">
-        <v>Trạng thái "Đang tính" gộp PENDING+RUNNING</v>
+        <v>Kiểm tra hiển thị đúng trạng thái "Đang tính" gộp thành công cho cả 2 giá trị PENDING và RUNNING</v>
       </c>
       <c r="E75" t="str">
         <v>Run đang PENDING hoặc RUNNING</v>
@@ -2650,7 +2650,7 @@
         <v>High</v>
       </c>
       <c r="D76" t="str">
-        <v>Polling tự động mỗi 5s khi Đang tính</v>
+        <v>Kiểm tra polling tự động đúng chu kỳ 5s và hội tụ đúng công thức BQGQ với dữ liệu phiếu tự tham chiếu</v>
       </c>
       <c r="E76" t="str">
         <v>Run đang chạy; Pre-condition: có mã với phiếu "Nhập hàng bán bị trả lại" tự tham chiếu Xuất bán cùng kỳ (setup: tạo phiếu Nhập mua → phiếu Xuất bán từ mã đó → phiếu Nhập hàng bán bị trả lại tham chiếu phiếu Xuất bán trên, "Tự nhập giá" để trống)</v>
@@ -2680,7 +2680,7 @@
         <v>High</v>
       </c>
       <c r="D77" t="str">
-        <v>Polling dừng khi SUCCEEDED</v>
+        <v>Kiểm tra dừng polling thành công khi run chuyển trạng thái SUCCEEDED</v>
       </c>
       <c r="E77" t="str">
         <v>Run chuyển SUCCEEDED</v>
@@ -2711,7 +2711,7 @@
         <v>High</v>
       </c>
       <c r="D78" t="str">
-        <v>Polling dừng khi COMPLETED_WITH_ERRORS</v>
+        <v>Kiểm tra dừng polling thành công khi run chuyển trạng thái COMPLETED_WITH_ERRORS</v>
       </c>
       <c r="E78" t="str">
         <v>Run chuyển có lỗi</v>
@@ -2741,7 +2741,7 @@
         <v>High</v>
       </c>
       <c r="D79" t="str">
-        <v>Bảng chi tiết đúng 11 cột</v>
+        <v>Kiểm tra hiển thị đúng 11 cột bảng chi tiết với dữ liệu run có items</v>
       </c>
       <c r="E79" t="str">
         <v>Run có items</v>
@@ -2770,7 +2770,7 @@
         <v>High</v>
       </c>
       <c r="D80" t="str">
-        <v>Dòng Tổng dùng aggregates BE</v>
+        <v>Kiểm tra dòng Tổng giữ nguyên giá trị aggregates BE thành công khi đổi filter trạng thái</v>
       </c>
       <c r="E80" t="str">
         <v>Bảng có filter/pagination áp dụng</v>
@@ -2800,7 +2800,7 @@
         <v>High</v>
       </c>
       <c r="D81" t="str">
-        <v>Mã lỗi hiển thị đúng badge + lý do</v>
+        <v>Kiểm tra hiển thị đúng badge và lý do lỗi "Do tồn âm" với dữ liệu mã lỗi NEGATIVE_STOCK</v>
       </c>
       <c r="E81" t="str">
         <v>Run có ≥1 mã lỗi "Do tồn âm"</v>
@@ -2831,7 +2831,7 @@
         <v>High</v>
       </c>
       <c r="D82" t="str">
-        <v>Mã lỗi "Do sự cố hệ thống" (SYSTEM_ERROR)</v>
+        <v>Kiểm tra hiển thị đúng lý do lỗi "Do sự cố hệ thống" với dữ liệu mã lỗi SYSTEM_ERROR</v>
       </c>
       <c r="E82" t="str">
         <v>Job nền bị gián đoạn/hết retry trước khi tính tới 1 mã (cần phối hợp giả lập gián đoạn — khó tái tạo bằng thao tác UI thông thường)</v>
@@ -2861,7 +2861,7 @@
         <v>High</v>
       </c>
       <c r="D83" t="str">
-        <v>Mẫu số=0 (không tồn đầu, không nhập trong kỳ) → đơn giá=0</v>
+        <v>Kiểm tra tính đơn giá bình quân = 0 thành công với dữ liệu mã PN-18903 không có tồn đầu/nhập trong kỳ</v>
       </c>
       <c r="E83" t="str">
         <v>Mã PN-18903 không có phiếu nhập/xuất nào trong kỳ, không có tồn đầu</v>
@@ -2892,7 +2892,7 @@
         <v>High</v>
       </c>
       <c r="D84" t="str">
-        <v>Giá bình quân hiển thị đúng 2 chữ số thập phân</v>
+        <v>Kiểm tra hiển thị đúng giá bình quân làm tròn 2 chữ số thập phân với dữ liệu kết quả thập phân dài</v>
       </c>
       <c r="E84" t="str">
         <v>Mã có kết quả tính ra số thập phân dài (vd 3 chữ số)</v>
@@ -2922,7 +2922,7 @@
         <v>High</v>
       </c>
       <c r="D85" t="str">
-        <v>Mở Detail với runId không tồn tại</v>
+        <v>Kiểm tra redirect về LIST thành công với dữ liệu runId=99999 không tồn tại</v>
       </c>
       <c r="E85" t="str">
         <v>runId=99999 không có</v>
@@ -2952,7 +2952,7 @@
         <v>High</v>
       </c>
       <c r="D86" t="str">
-        <v>Feature flag OFF</v>
+        <v>Kiểm tra chặn truy cập màn Detail thành công khi feature flag Inventory:InventoryV2 đang OFF</v>
       </c>
       <c r="E86" t="str">
         <v>Flag Inventory:InventoryV2 OFF</v>
@@ -3010,7 +3010,7 @@
         <v>Medium</v>
       </c>
       <c r="D88" t="str">
-        <v>Filter search (mã/tên) — client-side</v>
+        <v>Kiểm tra filter search (mã/tên) client-side thành công với từ khóa "PN-189"</v>
       </c>
       <c r="E88" t="str">
         <v>Bảng có nhiều mã</v>
@@ -3040,7 +3040,7 @@
         <v>Medium</v>
       </c>
       <c r="D89" t="str">
-        <v>Filter dropdown "Trạng thái"</v>
+        <v>Kiểm tra filter dropdown "Trạng thái" thành công với giá trị "Lỗi"</v>
       </c>
       <c r="E89" t="str">
         <v>Bảng có mã Đã tính + Lỗi</v>
@@ -3069,7 +3069,7 @@
         <v>Medium</v>
       </c>
       <c r="D90" t="str">
-        <v>Kết hợp search + dropdown trạng thái</v>
+        <v>Kiểm tra kết hợp filter search + dropdown "Trạng thái" thành công theo điều kiện AND</v>
       </c>
       <c r="E90" t="str">
         <v>—</v>
@@ -3127,7 +3127,7 @@
         <v>Medium</v>
       </c>
       <c r="D92" t="str">
-        <v>RunInfoGrid dùng cặp label-value chuẩn a11y</v>
+        <v>Kiểm tra RunInfoGrid dùng đúng cặp label-value chuẩn a11y</v>
       </c>
       <c r="E92" t="str">
         <v>—</v>
@@ -3156,7 +3156,7 @@
         <v>Medium</v>
       </c>
       <c r="D93" t="str">
-        <v>Bảng chi tiết &amp; dòng Tổng đúng semantic</v>
+        <v>Kiểm tra bảng chi tiết và dòng Tổng đúng semantic HTML</v>
       </c>
       <c r="E93" t="str">
         <v>—</v>
@@ -3185,7 +3185,7 @@
         <v>Medium</v>
       </c>
       <c r="D94" t="str">
-        <v>Badge "Lỗi" không chỉ dựa màu</v>
+        <v>Kiểm tra badge "Lỗi" hiển thị đúng kèm text, không chỉ dựa vào màu</v>
       </c>
       <c r="E94" t="str">
         <v>Có dòng lỗi</v>
@@ -3214,7 +3214,7 @@
         <v>Medium</v>
       </c>
       <c r="D95" t="str">
-        <v>Nút Recalc loading aria-busy</v>
+        <v>Kiểm tra nút Recalc có đúng thuộc tính aria-busy khi đang loading</v>
       </c>
       <c r="E95" t="str">
         <v>Bấm nút Recalc</v>
@@ -3243,7 +3243,7 @@
         <v>Medium</v>
       </c>
       <c r="D96" t="str">
-        <v>Empty state khi filter không khớp</v>
+        <v>Kiểm tra hiển thị empty state thành công khi filter search không khớp từ khóa "ZZZ-000"</v>
       </c>
       <c r="E96" t="str">
         <v>Search từ khóa không tồn tại</v>
@@ -3301,7 +3301,7 @@
         <v>High</v>
       </c>
       <c r="D98" t="str">
-        <v>garage-owner thấy đủ RunInfoGrid + bảng + 2 nút Recalc</v>
+        <v>Kiểm tra phân quyền hiển thị đầy đủ RunInfoGrid, bảng và 2 nút Recalc thành công cho vai trò garage-owner</v>
       </c>
       <c r="E98" t="str">
         <v>Tài khoản garage-owner</v>
@@ -3330,7 +3330,7 @@
         <v>High</v>
       </c>
       <c r="D99" t="str">
-        <v>accountant thấy giống garage-owner</v>
+        <v>Kiểm tra phân quyền hiển thị đầy đủ thành công giống garage-owner cho vai trò accountant</v>
       </c>
       <c r="E99" t="str">
         <v>Tài khoản accountant</v>
@@ -3388,7 +3388,7 @@
         <v>High</v>
       </c>
       <c r="D101" t="str">
-        <v>Mã SUCCEEDED khớp báo cáo Stock V2</v>
+        <v>Kiểm tra giá trị Giá bình quân khớp đúng báo cáo Stock V2 với dữ liệu mã PN-18901 SUCCEEDED</v>
       </c>
       <c r="E101" t="str">
         <v>Run SUCCEEDED, mã PN-18901</v>
@@ -3417,7 +3417,7 @@
         <v>High</v>
       </c>
       <c r="D102" t="str">
-        <v>Cross-wave: phiếu Xuất bán hiển thị đúng giá vốn mới sau PRC</v>
+        <v>Kiểm tra phiếu Xuất bán hiển thị đúng giá vốn mới thành công sau khi PRC tính giá (cross-wave)</v>
       </c>
       <c r="E102" t="str">
         <v>Mã đã PRC tính giá thành công, có phiếu Xuất bán trong kỳ (thuộc W05, ngoài phạm vi wave 6)</v>
@@ -3446,7 +3446,7 @@
         <v>High</v>
       </c>
       <c r="D103" t="str">
-        <v>Cross-wave: phiếu "Nhập hàng bán bị trả lại" hiển thị đúng giá kế thừa</v>
+        <v>Kiểm tra phiếu "Nhập hàng bán bị trả lại" hiển thị đúng giá kế thừa thành công từ phiếu Xuất bán gốc (cross-wave)</v>
       </c>
       <c r="E103" t="str">
         <v>Có phiếu trả hàng kế thừa giá từ phiếu Xuất bán gốc đã PRC tính</v>
@@ -3475,7 +3475,7 @@
         <v>High</v>
       </c>
       <c r="D104" t="str">
-        <v>Disable 2 nút Recalc khi run đang PENDING/RUNNING</v>
+        <v>Kiểm tra disable 2 nút Recalc thành công khi run đang PENDING/RUNNING</v>
       </c>
       <c r="E104" t="str">
         <v>Run đang chạy</v>
@@ -3504,7 +3504,7 @@
         <v>High</v>
       </c>
       <c r="D105" t="str">
-        <v>Ẩn/disable "Tính lại mã lỗi" khi không có mã lỗi</v>
+        <v>Kiểm tra ẩn/disable nút "Tính lại mã lỗi" thành công khi run không có mã lỗi</v>
       </c>
       <c r="E105" t="str">
         <v>Run SUCCEEDED hoàn toàn (itemsErrorCount=0)</v>
@@ -3562,7 +3562,7 @@
         <v>High</v>
       </c>
       <c r="D107" t="str">
-        <v>Bấm "Tính lại toàn bộ"</v>
+        <v>Kiểm tra RECALC scope ALL thành công khi bấm "Tính lại toàn bộ"</v>
       </c>
       <c r="E107" t="str">
         <v>Run có kết quả cũ</v>
@@ -3593,7 +3593,7 @@
         <v>High</v>
       </c>
       <c r="D108" t="str">
-        <v>Bấm "Tính lại mã lỗi"</v>
+        <v>Kiểm tra RECALC scope ERROR_ONLY thành công khi bấm "Tính lại mã lỗi"</v>
       </c>
       <c r="E108" t="str">
         <v>Run có ≥1 mã lỗi</v>
@@ -3623,7 +3623,7 @@
         <v>High</v>
       </c>
       <c r="D109" t="str">
-        <v>Response affectedSubsequentPeriods non-empty</v>
+        <v>Kiểm tra hiển thị toast cảnh báo thành công với dữ liệu response affectedSubsequentPeriods non-empty</v>
       </c>
       <c r="E109" t="str">
         <v>Kỳ sau đã tính</v>
@@ -3652,7 +3652,7 @@
         <v>High</v>
       </c>
       <c r="D110" t="str">
-        <v>RECALC khi kỳ đã đóng</v>
+        <v>Kiểm tra RECALC thất bại với dữ liệu Kỳ kế toán đã đóng</v>
       </c>
       <c r="E110" t="str">
         <v>Kỳ đã đóng</v>
@@ -3681,7 +3681,7 @@
         <v>High</v>
       </c>
       <c r="D111" t="str">
-        <v>RECALC khi đang có job chạy cùng kỳ+kho</v>
+        <v>Kiểm tra RECALC thất bại khi đang có job RUNNING cùng kỳ+kho</v>
       </c>
       <c r="E111" t="str">
         <v>Job khác đang RUNNING cùng kỳ+kho</v>
@@ -3710,7 +3710,7 @@
         <v>High</v>
       </c>
       <c r="D112" t="str">
-        <v>Double-click nút Recalc</v>
+        <v>Kiểm tra chặn tạo trùng request thành công khi double-click nút Recalc</v>
       </c>
       <c r="E112" t="str">
         <v>—</v>
@@ -3739,7 +3739,7 @@
         <v>High</v>
       </c>
       <c r="D113" t="str">
-        <v>Mở lại kỳ đã đóng rồi RECALC</v>
+        <v>Kiểm tra RECALC thành công với dữ liệu kỳ vừa được mở lại</v>
       </c>
       <c r="E113" t="str">
         <v>Kỳ vừa mở lại</v>
@@ -3798,7 +3798,7 @@
         <v>Medium</v>
       </c>
       <c r="D115" t="str">
-        <v>Label "Tính lại  toàn bộ" đúng verbatim (2 khoảng trắng)</v>
+        <v>Kiểm tra hiển thị đúng label "Tính lại  toàn bộ" verbatim theo Figma (2 khoảng trắng)</v>
       </c>
       <c r="E115" t="str">
         <v>—</v>
@@ -3827,7 +3827,7 @@
         <v>Medium</v>
       </c>
       <c r="D116" t="str">
-        <v>Label "Tính lại mã lỗi " đúng verbatim</v>
+        <v>Kiểm tra hiển thị đúng label "Tính lại mã lỗi " verbatim theo Figma</v>
       </c>
       <c r="E116" t="str">
         <v>—</v>
@@ -3856,7 +3856,7 @@
         <v>Medium</v>
       </c>
       <c r="D117" t="str">
-        <v>2 nút disable đồng thời khi loading</v>
+        <v>Kiểm tra disable đồng thời cả 2 nút Recalc thành công khi đang loading</v>
       </c>
       <c r="E117" t="str">
         <v>Bấm 1 nút</v>
@@ -3885,7 +3885,7 @@
         <v>Medium</v>
       </c>
       <c r="D118" t="str">
-        <v>Dialog lỗi trap focus + Escape</v>
+        <v>Kiểm tra đóng dialog lỗi thành công và trả focus đúng khi nhấn Escape</v>
       </c>
       <c r="E118" t="str">
         <v>Dialog lỗi đang mở</v>
@@ -3943,7 +3943,7 @@
         <v>High</v>
       </c>
       <c r="D120" t="str">
-        <v>garage-owner bấm được cả 2 nút</v>
+        <v>Kiểm tra phân quyền bấm được cả 2 nút Recalc thành công cho vai trò garage-owner</v>
       </c>
       <c r="E120" t="str">
         <v>Tài khoản garage-owner</v>
@@ -3972,7 +3972,7 @@
         <v>High</v>
       </c>
       <c r="D121" t="str">
-        <v>accountant bấm được cả 2 nút</v>
+        <v>Kiểm tra phân quyền bấm được cả 2 nút Recalc thành công cho vai trò accountant</v>
       </c>
       <c r="E121" t="str">
         <v>Tài khoản accountant</v>
@@ -4030,7 +4030,7 @@
         <v>High</v>
       </c>
       <c r="D123" t="str">
-        <v>Run mới có source_run_id trỏ đúng run gốc</v>
+        <v>Kiểm tra run mới có source_run_id trỏ đúng run gốc thành công sau khi RECALC</v>
       </c>
       <c r="E123" t="str">
         <v>Sau RECALC</v>
@@ -4059,7 +4059,7 @@
         <v>High</v>
       </c>
       <c r="D124" t="str">
-        <v>Scope ERROR_ONLY giữ nguyên mã "Đã tính"</v>
+        <v>Kiểm tra RECALC scope ERROR_ONLY giữ nguyên kết quả mã "Đã tính" thành công</v>
       </c>
       <c r="E124" t="str">
         <v>Run có mã Đã tính + mã Lỗi</v>
@@ -4088,7 +4088,7 @@
         <v>High</v>
       </c>
       <c r="D125" t="str">
-        <v>Kết quả RECALC cập nhật đúng ở Stock V2 Reports</v>
+        <v>Kiểm tra báo cáo Stock V2 Reports cập nhật đúng giá trị thành công sau khi RECALC</v>
       </c>
       <c r="E125" t="str">
         <v>Sau RECALC thành công</v>
@@ -4117,7 +4117,7 @@
         <v>High</v>
       </c>
       <c r="D126" t="str">
-        <v>2 request RECALC/CREATE gần đồng thời cùng kỳ+kho</v>
+        <v>Kiểm tra chặn concurrency thành công khi 2 request RECALC/CREATE gần đồng thời cùng kỳ+kho</v>
       </c>
       <c r="E126" t="str">
         <v>Mở 2 tab, cùng điền form giống nhau (best-effort thủ công — race condition không đảm bảo chính xác 100% qua thao tác tay, khuyến nghị bổ sung automation/integration test riêng)</v>
@@ -4177,7 +4177,7 @@
         <v>High</v>
       </c>
       <c r="D128" t="str">
-        <v>Click icon Xóa mở dialog đúng nội dung</v>
+        <v>Kiểm tra mở dialog xác nhận xóa đúng nội dung thành công khi click icon "Xóa"</v>
       </c>
       <c r="E128" t="str">
         <v>Bảng LIST có data</v>
@@ -4206,7 +4206,7 @@
         <v>High</v>
       </c>
       <c r="D129" t="str">
-        <v>Xác nhận xóa (kỳ mở, log terminal)</v>
+        <v>Kiểm tra xóa log thành công với dữ liệu kỳ mở và log ở trạng thái terminal (SUCCEEDED)</v>
       </c>
       <c r="E129" t="str">
         <v>Log SUCCEEDED, kỳ mở</v>
@@ -4237,7 +4237,7 @@
         <v>High</v>
       </c>
       <c r="D130" t="str">
-        <v>Hủy — đóng dialog không xóa</v>
+        <v>Kiểm tra đóng dialog xác nhận thành công khi bấm "Hủy", không thực hiện xóa</v>
       </c>
       <c r="E130" t="str">
         <v>—</v>
@@ -4266,7 +4266,7 @@
         <v>High</v>
       </c>
       <c r="D131" t="str">
-        <v>Escape — đóng dialog không xóa</v>
+        <v>Kiểm tra đóng dialog xác nhận thành công khi nhấn Escape, không thực hiện xóa</v>
       </c>
       <c r="E131" t="str">
         <v>—</v>
@@ -4295,7 +4295,7 @@
         <v>High</v>
       </c>
       <c r="D132" t="str">
-        <v>Xóa khi kỳ đã đóng</v>
+        <v>Kiểm tra xóa log thất bại với dữ liệu Kỳ kế toán đã đóng</v>
       </c>
       <c r="E132" t="str">
         <v>Log thuộc kỳ đã đóng</v>
@@ -4324,7 +4324,7 @@
         <v>High</v>
       </c>
       <c r="D133" t="str">
-        <v>Xóa khi log đang "Đang tính"</v>
+        <v>Kiểm tra xóa log thất bại với dữ liệu log đang ở trạng thái "Đang tính" (PENDING/RUNNING)</v>
       </c>
       <c r="E133" t="str">
         <v>Log status=PENDING/RUNNING</v>
@@ -4353,7 +4353,7 @@
         <v>High</v>
       </c>
       <c r="D134" t="str">
-        <v>Xóa thành công — giá vốn không rollback</v>
+        <v>Kiểm tra xóa log thành công và giá vốn phiếu xuất không bị rollback</v>
       </c>
       <c r="E134" t="str">
         <v>Log SUCCEEDED đã cập nhật giá vốn</v>
@@ -4412,7 +4412,7 @@
         <v>N/A</v>
       </c>
       <c r="D136" t="str">
-        <v>Không có field cần validate</v>
+        <v>Kiểm tra dialog xác nhận xóa không phát sinh field cần validate (N/A)</v>
       </c>
       <c r="E136" t="str">
         <v>—</v>
@@ -4470,7 +4470,7 @@
         <v>Medium</v>
       </c>
       <c r="D138" t="str">
-        <v>Dialog width 441px, bo góc vuông</v>
+        <v>Kiểm tra dialog xác nhận xóa đúng kích thước 441px và bo góc vuông</v>
       </c>
       <c r="E138" t="str">
         <v>Dialog xác nhận đang mở</v>
@@ -4499,7 +4499,7 @@
         <v>Medium</v>
       </c>
       <c r="D139" t="str">
-        <v>Title luôn màu đen dù biến thể nào</v>
+        <v>Kiểm tra title dialog luôn hiển thị màu đen với mọi biến thể nội dung</v>
       </c>
       <c r="E139" t="str">
         <v>Dialog "Không thể xóa" đang mở</v>
@@ -4528,7 +4528,7 @@
         <v>Medium</v>
       </c>
       <c r="D140" t="str">
-        <v>Nút loading khi đang chờ mutation</v>
+        <v>Kiểm tra hiển thị loading state thành công cho nút "Xác nhận xoá" khi đang chờ mutation</v>
       </c>
       <c r="E140" t="str">
         <v>Bấm "Xác nhận xoá"</v>
@@ -4557,7 +4557,7 @@
         <v>Medium</v>
       </c>
       <c r="D141" t="str">
-        <v>KHÔNG hiển thị mã lỗi kỹ thuật ra UI</v>
+        <v>Kiểm tra không hiển thị mã lỗi kỹ thuật ra UI tại dialog chặn xóa</v>
       </c>
       <c r="E141" t="str">
         <v>Dialog chặn đang mở</v>
@@ -4586,7 +4586,7 @@
         <v>Medium</v>
       </c>
       <c r="D142" t="str">
-        <v>Nút xác nhận đúng label "Xác nhận xoá"</v>
+        <v>Kiểm tra hiển thị đúng label "Xác nhận xoá" verbatim theo Figma</v>
       </c>
       <c r="E142" t="str">
         <v>—</v>
@@ -4644,7 +4644,7 @@
         <v>High</v>
       </c>
       <c r="D144" t="str">
-        <v>garage-owner thao tác xóa đầy đủ</v>
+        <v>Kiểm tra phân quyền thao tác xóa thành công cho vai trò garage-owner</v>
       </c>
       <c r="E144" t="str">
         <v>Tài khoản garage-owner</v>
@@ -4673,7 +4673,7 @@
         <v>High</v>
       </c>
       <c r="D145" t="str">
-        <v>accountant thao tác xóa đầy đủ</v>
+        <v>Kiểm tra phân quyền thao tác xóa thành công cho vai trò accountant</v>
       </c>
       <c r="E145" t="str">
         <v>Tài khoản accountant</v>
@@ -4731,7 +4731,7 @@
         <v>High</v>
       </c>
       <c r="D147" t="str">
-        <v>Sau xóa, dữ liệu Stock V2 Reports không đổi (đúng thiết kế không rollback)</v>
+        <v>Kiểm tra dữ liệu Stock V2 Reports giữ nguyên không đổi thành công sau khi xóa log (đúng thiết kế không rollback)</v>
       </c>
       <c r="E147" t="str">
         <v>Đã xóa 1 log SUCCEEDED</v>

</xml_diff>